<commit_message>
Refresh valuation to FY2026 actuals and 10/26/2026 inputs
Roll the forecast to FY2027E-FY2031E with FY2026 actuals, current price,
10Y yield and beta. Add stub-period discounting, count short-term
investments as cash, fix the terminal value growing FCFF by (1+g) twice,
and make the sensitivity grid and summary live formulas. The April model
is kept in excel/archive and tagged v1-apr2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/MSFT_DCF_Model.xlsx
+++ b/excel/MSFT_DCF_Model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/masontrinkner/Python/Python:Excel Project/msft-dcf-valuation/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/masontrinkner/ClaudeCode/msft-dcf-valuation/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D8C29C0-0147-E241-9DDC-2458CC1F2F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEC767A-91AB-A347-BC7D-97B233354D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17420" yWindow="780" windowWidth="16780" windowHeight="21460" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,12 +21,6 @@
     <sheet name="Sensitivity" sheetId="6" r:id="rId6"/>
     <sheet name="Summary" sheetId="7" r:id="rId7"/>
   </sheets>
-  <definedNames>
-    <definedName name="ebit_margin_pct">Historicals!$G$11</definedName>
-    <definedName name="gross_margin_pct">Historicals!$F$11</definedName>
-    <definedName name="latest_cash_cell">Historicals!$M$9</definedName>
-    <definedName name="latest_debt_cell">Historicals!$L$9</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -45,7 +39,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="138">
+  <si>
+    <t>MSFT DCF Model - Summary</t>
+  </si>
+  <si>
+    <t>Values in USD - fiscal year ending June 30</t>
+  </si>
+  <si>
+    <t>COMPANY OVERVIEW</t>
+  </si>
+  <si>
+    <t>Company | Microsoft Corporation</t>
+  </si>
+  <si>
+    <t>Sector | Technology</t>
+  </si>
+  <si>
+    <t>VALUATION SUMMARY</t>
+  </si>
+  <si>
+    <t>Recommendation | Small long position, long-term horizon</t>
+  </si>
+  <si>
+    <t>KEY ASSUMPTIONS</t>
+  </si>
+  <si>
+    <t>Projection Period | FY2027E - FY2031E</t>
+  </si>
+  <si>
+    <t>INVESTMENT THESIS</t>
+  </si>
+  <si>
+    <t>Upside | Copilot/Azure AI adoption faster than modeled</t>
+  </si>
+  <si>
+    <t>Downside | AI CapEx doesn't translate to revenue growth</t>
+  </si>
+  <si>
+    <t>View | Market pricing in more optimism than base case justifies</t>
+  </si>
   <si>
     <t>MSFT — Historical Financials (yfinance · Python-Generated)</t>
   </si>
@@ -95,6 +128,12 @@
     <t>Net WC</t>
   </si>
   <si>
+    <t>Cash + ST Inv</t>
+  </si>
+  <si>
+    <t>3yr Average:</t>
+  </si>
+  <si>
     <t>MSFT — Company Profile (via yfinance)</t>
   </si>
   <si>
@@ -128,338 +167,303 @@
     <t>52w Low</t>
   </si>
   <si>
+    <t>As of</t>
+  </si>
+  <si>
+    <t>10/26/2026 close (Yahoo Finance)</t>
+  </si>
+  <si>
     <t>MSFT DCF Model - Assumptions</t>
   </si>
   <si>
+    <t>Values in USD - fiscal year ending June 30 | Data Pulled From Alpha Spread, StockTitan, CNBC</t>
+  </si>
+  <si>
+    <t>CapEx modeled as a glide path rather than flat assumption. FY2026A came in at 34.9% of revenue (vs 30% modeled in April), so the April glide path is shifted one year later.</t>
+  </si>
+  <si>
+    <t>REVENUE GROWTH ASSUMPTIONS</t>
+  </si>
+  <si>
+    <t>Revenue Growth - FY2027E</t>
+  </si>
+  <si>
+    <t>Apr-2026 FY2027E assumption (Alpha Spread 3yr CAGR); FY2026A was 17.8%</t>
+  </si>
+  <si>
+    <t>Revenue Growth - FY2028E</t>
+  </si>
+  <si>
+    <t>Interpolation</t>
+  </si>
+  <si>
+    <t>Revenue Growth - FY2029E</t>
+  </si>
+  <si>
+    <t>Revenue Growth - FY2030E</t>
+  </si>
+  <si>
+    <t>Revenue Growth - FY2031E</t>
+  </si>
+  <si>
+    <t>Interpolation (extends taper one year)</t>
+  </si>
+  <si>
+    <t>MARGIN ASSUMPTIONS</t>
+  </si>
+  <si>
+    <t>Gross Margin %</t>
+  </si>
+  <si>
+    <t>FY2026 Historicals</t>
+  </si>
+  <si>
+    <t>EBIT Margin %</t>
+  </si>
+  <si>
+    <t>FY2026 actual effective rate</t>
+  </si>
+  <si>
+    <t>CASH FLOW ASSUMPTIONS</t>
+  </si>
+  <si>
+    <t>D&amp;A as % of Revenue</t>
+  </si>
+  <si>
+    <t>3yr avg FY2024-FY2026</t>
+  </si>
+  <si>
+    <t>CapEx as % of Revenue (2027E-2031E)</t>
+  </si>
+  <si>
+    <t>FY2026A 34.9% (Q4 FY2026 alone 39.8%); April glide path (30/24/18/14/11) shifted one year; pre-AI steady state ~13% (FY2023)</t>
+  </si>
+  <si>
+    <t>Change NWC as % of Rev Change</t>
+  </si>
+  <si>
+    <t>3yr avg FY2023-FY2025</t>
+  </si>
+  <si>
+    <t>WACC INPUTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk-Free Rate </t>
+  </si>
+  <si>
+    <t>10Y Treasury yield, 10/26/26</t>
+  </si>
+  <si>
+    <t>Equity Risk Premium</t>
+  </si>
+  <si>
+    <t>Alpha Spread</t>
+  </si>
+  <si>
+    <t>Yahoo Finance, 10/26/26 (was 1.107 in April)</t>
+  </si>
+  <si>
+    <t>Cost of Equity</t>
+  </si>
+  <si>
+    <t>CAPM</t>
+  </si>
+  <si>
+    <t>Pre-tax Cost of Debt</t>
+  </si>
+  <si>
+    <t>Aprox MSFT bond yield, Alpha Spread</t>
+  </si>
+  <si>
+    <t>After-tax Cost of Debt</t>
+  </si>
+  <si>
+    <t>Pre-tax cost of debt * (1 - tax rate)</t>
+  </si>
+  <si>
+    <t>Debt Weight</t>
+  </si>
+  <si>
+    <t>Market value: total debt / (total debt + market cap)</t>
+  </si>
+  <si>
+    <t>Equity Rate</t>
+  </si>
+  <si>
+    <t>1 - Debt Weight</t>
+  </si>
+  <si>
+    <t>WACC</t>
+  </si>
+  <si>
+    <t>(Equity Rate * Cost of Equity) + (Debt Weight * After-tax Cost of Debt)</t>
+  </si>
+  <si>
+    <t>TERMINAL VALUE INPUTS</t>
+  </si>
+  <si>
+    <t>Terminal Growth Rate</t>
+  </si>
+  <si>
+    <t>Long-run nominal GDP</t>
+  </si>
+  <si>
+    <t>SHARES &amp; PRICE</t>
+  </si>
+  <si>
+    <t>yfinance</t>
+  </si>
+  <si>
+    <t>Current Stock Price</t>
+  </si>
+  <si>
+    <t>Yahoo Finance close, 10/26/26</t>
+  </si>
+  <si>
+    <t>VALUATION TIMING</t>
+  </si>
+  <si>
+    <t>Valuation Date</t>
+  </si>
+  <si>
+    <t>Price date</t>
+  </si>
+  <si>
+    <t>FY2027 Year End</t>
+  </si>
+  <si>
+    <t>Fiscal year ends June 30</t>
+  </si>
+  <si>
+    <t>Stub Fraction (FY2027E)</t>
+  </si>
+  <si>
+    <t>Share of FY2027E cash flow still ahead of the valuation date</t>
+  </si>
+  <si>
     <t>MSFT DCF Model - Forecast</t>
   </si>
   <si>
+    <t>FY2022</t>
+  </si>
+  <si>
+    <t>FY2023</t>
+  </si>
+  <si>
+    <t>FY2024</t>
+  </si>
+  <si>
+    <t>FY2025</t>
+  </si>
+  <si>
+    <t>FY2026</t>
+  </si>
+  <si>
+    <t>FY2027E</t>
+  </si>
+  <si>
+    <t>FY2028E</t>
+  </si>
+  <si>
+    <t>FY2029E</t>
+  </si>
+  <si>
+    <t>FY2030E</t>
+  </si>
+  <si>
+    <t>FY2031E</t>
+  </si>
+  <si>
+    <t>Revenue Growth %</t>
+  </si>
+  <si>
+    <t>Free Cash Flow Build</t>
+  </si>
+  <si>
+    <t>NOPAT (EBIT after Tax)</t>
+  </si>
+  <si>
+    <t>Plus: D&amp;A</t>
+  </si>
+  <si>
+    <t>Less: CapEx</t>
+  </si>
+  <si>
+    <t>Less: Change in NWC</t>
+  </si>
+  <si>
+    <t>FCFF</t>
+  </si>
+  <si>
     <t>MSFT DCF Model - DCF</t>
   </si>
   <si>
+    <t>Forecast Year</t>
+  </si>
+  <si>
+    <t>Discount Period</t>
+  </si>
+  <si>
+    <t>FCFF (FY2027E pro-rated to stub)</t>
+  </si>
+  <si>
+    <t>Discount Factor</t>
+  </si>
+  <si>
+    <t>PV of FCFF</t>
+  </si>
+  <si>
+    <t>Sum of PV (FCFF)</t>
+  </si>
+  <si>
+    <t>Terminal Year FCFF (FY2032E)</t>
+  </si>
+  <si>
+    <t>Terminal Value</t>
+  </si>
+  <si>
+    <t>PV of Terminal Value</t>
+  </si>
+  <si>
+    <t>Enterprise Value</t>
+  </si>
+  <si>
+    <t>Less: Total Debt</t>
+  </si>
+  <si>
+    <t>Plus: Cash &amp; Short-Term Investments</t>
+  </si>
+  <si>
+    <t>Equity Value</t>
+  </si>
+  <si>
+    <t>Intrinsic Value Per Share</t>
+  </si>
+  <si>
+    <t>Implied Upside / Downside</t>
+  </si>
+  <si>
     <t>MSFT DCF Model - Sensitivity</t>
   </si>
   <si>
-    <t>MSFT DCF Model - Summary</t>
-  </si>
-  <si>
-    <t>Values in USD - fiscal year ending June 30</t>
-  </si>
-  <si>
-    <t>FY2021</t>
-  </si>
-  <si>
-    <t>FY2022</t>
-  </si>
-  <si>
-    <t>FY2023</t>
-  </si>
-  <si>
-    <t>FY2024</t>
-  </si>
-  <si>
-    <t>FY2025</t>
-  </si>
-  <si>
-    <t>FY2026E</t>
-  </si>
-  <si>
-    <t>FY2027E</t>
-  </si>
-  <si>
-    <t>FY2028E</t>
-  </si>
-  <si>
-    <t>FY2029E</t>
-  </si>
-  <si>
-    <t>FY2030E</t>
-  </si>
-  <si>
-    <t>REVENUE GROWTH ASSUMPTIONS</t>
-  </si>
-  <si>
-    <t>Revenue Growth - FY2026E</t>
-  </si>
-  <si>
-    <t>Revenue Growth - FY2027E</t>
-  </si>
-  <si>
-    <t>Revenue Growth - FY2028E</t>
-  </si>
-  <si>
-    <t>Revenue Growth - FY2029E</t>
-  </si>
-  <si>
-    <t>Revenue Growth - FY2030E</t>
-  </si>
-  <si>
-    <t>Gross Margin %</t>
-  </si>
-  <si>
-    <t>MARGIN ASSUMPTIONS</t>
-  </si>
-  <si>
-    <t>EBIT Margin %</t>
-  </si>
-  <si>
-    <t>CASH FLOW ASSUMPTIONS</t>
-  </si>
-  <si>
-    <t>D&amp;A as % of Revenue</t>
-  </si>
-  <si>
-    <t>Change NWC as % of Rev Change</t>
-  </si>
-  <si>
-    <t>WACC INPUTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk-Free Rate </t>
-  </si>
-  <si>
-    <t>Equity Risk Premium</t>
-  </si>
-  <si>
-    <t>Cost of Equity</t>
-  </si>
-  <si>
-    <t>Pre-tax Cost of Debt</t>
-  </si>
-  <si>
-    <t>After-tax Cost of Debt</t>
-  </si>
-  <si>
-    <t>Debt Weight</t>
-  </si>
-  <si>
-    <t>Equity Rate</t>
-  </si>
-  <si>
-    <t>WACC</t>
-  </si>
-  <si>
-    <t>TERMINAL VALUE INPUTS</t>
-  </si>
-  <si>
-    <t>Terminal Growth Rate</t>
-  </si>
-  <si>
-    <t>SHARES &amp; PRICE</t>
-  </si>
-  <si>
-    <t>Current Stock Price</t>
-  </si>
-  <si>
-    <t>CAPM</t>
-  </si>
-  <si>
-    <t>3yr Average:</t>
-  </si>
-  <si>
-    <t>Revenue Growth %</t>
-  </si>
-  <si>
-    <t>Free Cash Flow Build</t>
-  </si>
-  <si>
-    <t>NOPAT (EBIT after Tax)</t>
-  </si>
-  <si>
-    <t>Plus: D&amp;A</t>
-  </si>
-  <si>
-    <t>Less: CapEx</t>
-  </si>
-  <si>
-    <t>Less: Change in NWC</t>
-  </si>
-  <si>
-    <t>FCFF</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Forecast Year</t>
-  </si>
-  <si>
-    <t>Discount Factor</t>
-  </si>
-  <si>
-    <t>PV of FCFF</t>
-  </si>
-  <si>
-    <t>Terminal Year FCFF</t>
-  </si>
-  <si>
-    <t>Terminal Value</t>
-  </si>
-  <si>
-    <t>PV of Terminal Value</t>
-  </si>
-  <si>
-    <t>Enterprise Value</t>
-  </si>
-  <si>
-    <t>Less: Total Debt</t>
-  </si>
-  <si>
-    <t>Plus: Cash &amp; Equivalents</t>
-  </si>
-  <si>
-    <t>Equity Value</t>
-  </si>
-  <si>
-    <t>Discount Period</t>
-  </si>
-  <si>
-    <t>Sum of PV (FCFF)</t>
-  </si>
-  <si>
-    <t>Intrinsic Value Per Share</t>
-  </si>
-  <si>
-    <t>Implied Upside / Downside</t>
-  </si>
-  <si>
-    <t>Alpha Spread</t>
-  </si>
-  <si>
-    <t>yfinance</t>
-  </si>
-  <si>
-    <t>CapEx as % of Revenue (2026E-2030E)</t>
-  </si>
-  <si>
-    <t>Values in USD - fiscal year ending June 30 | Data Pulled From Alpha Spread, StockTitan, CNBC</t>
-  </si>
-  <si>
-    <t>CapEx modeled as a glide path rather than flat assumption. MSFT is at peak AI infrastructure spending (FY2026E - 30%). Spending will normalize as data center buildout matures</t>
-  </si>
-  <si>
-    <t>CNBC Q2 FY2026 Earnings Report</t>
-  </si>
-  <si>
-    <t>Alpha Spread 3yr Revenue CAGR</t>
-  </si>
-  <si>
-    <t>Interpolation</t>
-  </si>
-  <si>
-    <t>3yr avg FY2023-FY2025</t>
-  </si>
-  <si>
-    <t>CFO Hood Q1 FY2026 call; AI Buildout continues; Normalized; continued normalization; Pre-AI steady state (FY2023 was 13.3%</t>
-  </si>
-  <si>
-    <t>Alpha Spread, 4/19/26</t>
-  </si>
-  <si>
-    <t>yfinance; Alpha Spread shows 0.96</t>
-  </si>
-  <si>
-    <t>Aprox MSFT bond yield, Alpha Spread</t>
-  </si>
-  <si>
-    <t>Long-run nominal GDP</t>
-  </si>
-  <si>
-    <t>FY2025 Historicals</t>
-  </si>
-  <si>
-    <t>1 - Debt Weight</t>
-  </si>
-  <si>
-    <t>(Equity Rate * Cost of Equity) + (Debt Weight * After-tax Cost of Debt)</t>
-  </si>
-  <si>
-    <t>Pre-tax cost of debt * (1 - tax rate)</t>
-  </si>
-  <si>
-    <t>yfinance, 4/19/26</t>
-  </si>
-  <si>
-    <t>FY2025 actual effective rate</t>
-  </si>
-  <si>
     <t>Sensitivity Analysis: Intrinsic Value Per Share (USD)</t>
   </si>
   <si>
-    <t>WACC vs. Terminal Growth Rate | Base Case: $370.78 | Current Price: $424.16</t>
+    <t>TERMINAL GROWTH RATE →</t>
   </si>
   <si>
     <t>WACC ↓</t>
-  </si>
-  <si>
-    <t>TERMINAL GROWTH RATE →</t>
-  </si>
-  <si>
-    <t>COMPANY OVERVIEW</t>
-  </si>
-  <si>
-    <t>Company | Microsoft Corporation</t>
-  </si>
-  <si>
-    <t>Sector | Technology</t>
-  </si>
-  <si>
-    <t>Market Cap | $3,152.52T</t>
-  </si>
-  <si>
-    <t>Current Price | $424.16</t>
-  </si>
-  <si>
-    <t>Intrinsic Value Per Share | $380.14</t>
-  </si>
-  <si>
-    <t>Current Market Price | $424.16</t>
-  </si>
-  <si>
-    <t>Implied Upside / Downside | -10.38%</t>
-  </si>
-  <si>
-    <t>Recommendation | Small long position, long-term horizon</t>
-  </si>
-  <si>
-    <t>KEY ASSUMPTIONS</t>
-  </si>
-  <si>
-    <t>VALUATION SUMMARY</t>
-  </si>
-  <si>
-    <t>WACC | 8.80%</t>
-  </si>
-  <si>
-    <t>Terminal Growth Rate | 3.00%</t>
-  </si>
-  <si>
-    <t>FY2030E Revenue | $559.9B</t>
-  </si>
-  <si>
-    <t>Projection Period | FY2026E - FY2030E</t>
-  </si>
-  <si>
-    <t>INVESTMENT THESIS</t>
-  </si>
-  <si>
-    <t>Upside | Copilot/Azure AI adoption faster than modeled</t>
-  </si>
-  <si>
-    <t>Downside | AI CapEx doesn't translate to revenue growth</t>
-  </si>
-  <si>
-    <t>View | Market pricing in more optimism than base case justifies</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00,,,&quot;T&quot;"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -588,7 +592,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -622,6 +626,9 @@
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -971,7 +978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -981,77 +988,81 @@
     <col min="9" max="9" width="28.83203125" customWidth="1"/>
     <col min="10" max="10" width="23.5" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="14" width="16" customWidth="1"/>
+    <col min="12" max="13" width="16" customWidth="1"/>
+    <col min="14" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -1094,8 +1105,11 @@
       <c r="N5" s="4">
         <v>95749000000</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O5" s="4">
+        <v>130334000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1138,8 +1152,11 @@
       <c r="N6" s="4">
         <v>74602000000</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O6" s="4">
+        <v>104749000000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1162,7 +1179,7 @@
         <v>0.41772880636104098</v>
       </c>
       <c r="H7" s="5">
-        <v>0.18978625253328249</v>
+        <v>0.1897862525332826</v>
       </c>
       <c r="I7" s="4">
         <v>13861000000</v>
@@ -1182,8 +1199,11 @@
       <c r="N7" s="4">
         <v>80108000000</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O7" s="4">
+        <v>111256000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -1203,13 +1223,13 @@
         <v>0.69764443827971379</v>
       </c>
       <c r="G8" s="5">
-        <v>0.4464429957327371</v>
+        <v>0.44644299573273721</v>
       </c>
       <c r="H8" s="5">
-        <v>0.18231326597827191</v>
+        <v>0.18231326597827199</v>
       </c>
       <c r="I8" s="4">
-        <v>22287000000</v>
+        <v>20958000000</v>
       </c>
       <c r="J8" s="4">
         <v>44477000000</v>
@@ -1226,8 +1246,11 @@
       <c r="N8" s="4">
         <v>34448000000</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O8" s="4">
+        <v>75531000000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -1253,7 +1276,7 @@
         <v>0.1762964400980368</v>
       </c>
       <c r="I9" s="4">
-        <v>34153000000</v>
+        <v>29433000000</v>
       </c>
       <c r="J9" s="4">
         <v>64551000000</v>
@@ -1270,52 +1293,102 @@
       <c r="N9" s="4">
         <v>49913000000</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O9" s="4">
+        <v>94555000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="B10" s="4">
+        <v>331839000000</v>
+      </c>
+      <c r="C10" s="4">
+        <v>225465000000</v>
+      </c>
+      <c r="D10" s="4">
+        <v>155237000000</v>
+      </c>
+      <c r="E10" s="4">
+        <v>133749000000</v>
+      </c>
+      <c r="F10" s="5">
+        <v>0.67944093370580316</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0.46780818408927222</v>
+      </c>
+      <c r="H10" s="5">
+        <v>0.19396265985271249</v>
+      </c>
+      <c r="I10" s="4">
+        <v>38534000000</v>
+      </c>
+      <c r="J10" s="4">
+        <v>115948000000</v>
+      </c>
+      <c r="K10" s="4">
+        <v>66987000000</v>
+      </c>
+      <c r="L10" s="4">
+        <v>56826000000</v>
+      </c>
+      <c r="M10" s="4">
+        <v>20935000000</v>
+      </c>
+      <c r="N10" s="4">
+        <v>38885000000</v>
+      </c>
+      <c r="O10" s="4">
+        <v>76651000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="E11" s="12"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="H15" s="12"/>
       <c r="I15" s="11"/>
       <c r="J15" s="11"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="H16" s="12"/>
       <c r="I16" s="11" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="J16" s="11"/>
     </row>
     <row r="17" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H17" s="12">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="I17" s="11">
-        <f>I7/B7</f>
-        <v>6.5408300497841118E-2</v>
+        <f>I8/B8</f>
+        <v>8.5500281492481289E-2</v>
       </c>
       <c r="J17" s="11"/>
     </row>
     <row r="18" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H18" s="12">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="I18" s="11">
-        <f>I8/B8</f>
-        <v>9.0922071458294243E-2</v>
+        <f>I9/B9</f>
+        <v>0.10447459215402309</v>
       </c>
       <c r="J18" s="11"/>
     </row>
     <row r="19" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H19" s="12">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="I19" s="11">
-        <f>I9/B9</f>
-        <v>0.12122857832488534</v>
+        <f>I10/B10</f>
+        <v>0.11612257751499974</v>
       </c>
       <c r="J19" s="11"/>
     </row>
@@ -1324,11 +1397,11 @@
     </row>
     <row r="21" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H21" s="12" t="s">
-        <v>69</v>
+        <v>30</v>
       </c>
       <c r="I21" s="13">
-        <f>AVERAGE(I15, I16, I17, I18, I19)</f>
-        <v>9.2519650093673578E-2</v>
+        <f>AVERAGE(I17:I19)</f>
+        <v>0.10203248372050137</v>
       </c>
       <c r="J21" s="13"/>
     </row>
@@ -1345,80 +1418,88 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B5">
-        <v>1.107</v>
+        <v>1.099</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B6">
-        <v>7425629076</v>
+        <v>7425545491</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B7" s="20">
-        <v>3152517529600</v>
+        <v>3954845417472</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="B8">
-        <v>424.16</v>
+        <v>532.6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="B9">
-        <v>555.45000000000005</v>
+        <v>553.72</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B10">
-        <v>356.28</v>
+        <v>349.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1436,36 +1517,36 @@
     <col min="3" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C4" s="9"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B5" s="15">
-        <v>0.16700000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -1473,46 +1554,46 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B6" s="15">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B7" s="15">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B8" s="15">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B9" s="15">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1520,44 +1601,44 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B12" s="14">
-        <f>Historicals!F9</f>
-        <v>0.68823742386165188</v>
+        <f>Historicals!F10</f>
+        <v>0.67944093370580316</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B13" s="14">
-        <f>Historicals!G9</f>
-        <v>0.45621956240859851</v>
+        <f>Historicals!G10</f>
+        <v>0.46780818408927222</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B14" s="14">
-        <f>Historicals!H9</f>
-        <v>0.1762964400980368</v>
+        <f>Historicals!H10</f>
+        <v>0.19396265985271249</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="G14" s="14"/>
     </row>
@@ -1567,27 +1648,27 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B16" s="14"/>
       <c r="G16" s="16"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B17" s="14">
         <f>Historicals!I21</f>
-        <v>9.2519650093673578E-2</v>
+        <v>0.10203248372050137</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="G17" s="16"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="B18" s="15">
         <v>0.3</v>
@@ -1605,127 +1686,128 @@
         <v>0.11</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>101</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="B19" s="15">
         <v>0.03</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B22" s="15">
-        <v>4.3400000000000001E-2</v>
+        <v>4.99E-2</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>102</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B23" s="15">
         <v>4.1799999999999997E-2</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B24">
         <f>Profile!B5</f>
-        <v>1.107</v>
+        <v>1.099</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="B25" s="14">
         <f>B22+B24*B23</f>
-        <v>8.9672599999999991E-2</v>
+        <v>9.5838199999999998E-2</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="B26" s="15">
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B27" s="14">
         <f>B26*(1-B14)</f>
-        <v>2.8829624596568716E-2</v>
+        <v>2.8211306905155067E-2</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="B28" s="15">
-        <v>2.8000000000000001E-2</v>
+        <f>Historicals!L10/(Historicals!L10+Profile!B7)</f>
+        <v>1.4165168102379019E-2</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="B29" s="14">
         <f>1-B28</f>
-        <v>0.97199999999999998</v>
+        <v>0.985834831897621</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="B30" s="14">
         <f>B29*B25+B28*B27</f>
-        <v>8.7968996688703907E-2</v>
+        <v>9.4880253691069907E-2</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1733,52 +1815,88 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="B32" s="14"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="B33" s="15">
         <v>0.03</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B36">
         <f>Profile!B6</f>
-        <v>7425629076</v>
+        <v>7425545491</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="B37">
         <f>Profile!B8</f>
-        <v>424.16</v>
+        <v>532.6</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>110</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>94</v>
+      </c>
+      <c r="B40" s="25">
+        <v>46321</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="25">
+        <v>46568</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C42" s="10"/>
+      <c r="A42" t="s">
+        <v>98</v>
+      </c>
+      <c r="B42" s="26">
+        <f>(B41-B40)/365</f>
+        <v>0.67671232876712328</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>99</v>
+      </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
@@ -1826,574 +1944,576 @@
     <col min="11" max="11" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>33</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="H4" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="J4" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B5" s="10">
-        <f>Historicals!B5</f>
-        <v>168088000000</v>
-      </c>
-      <c r="C5" s="10">
         <f>Historicals!B6</f>
         <v>198270000000</v>
       </c>
-      <c r="D5" s="10">
+      <c r="C5" s="10">
         <f>Historicals!B7</f>
         <v>211915000000</v>
       </c>
-      <c r="E5" s="10">
+      <c r="D5" s="10">
         <f>Historicals!B8</f>
         <v>245122000000</v>
       </c>
-      <c r="F5" s="10">
+      <c r="E5" s="10">
         <f>Historicals!B9</f>
         <v>281724000000</v>
       </c>
+      <c r="F5" s="10">
+        <f>Historicals!B10</f>
+        <v>331839000000</v>
+      </c>
       <c r="G5" s="10">
         <f>F5*(1 + Assumptions!B5)</f>
-        <v>328771908000</v>
+        <v>388251630000</v>
       </c>
       <c r="H5" s="10">
         <f>G5*(1+Assumptions!B6)</f>
-        <v>384663132360</v>
+        <v>446489374499.99994</v>
       </c>
       <c r="I5" s="10">
         <f>H5*(1+Assumptions!B7)</f>
-        <v>442362602213.99994</v>
+        <v>504532993184.99988</v>
       </c>
       <c r="J5" s="10">
         <f>I5*(1+Assumptions!B8)</f>
-        <v>499869740501.81989</v>
+        <v>565076952367.19995</v>
       </c>
       <c r="K5" s="10">
         <f>J5*(1+Assumptions!B9)</f>
-        <v>559854109362.03833</v>
+        <v>627235417127.59204</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>77</v>
+        <v>111</v>
+      </c>
+      <c r="B6" s="10">
+        <f>B5/Historicals!B5-1</f>
+        <v>0.17956070629670173</v>
       </c>
       <c r="C6" s="10">
         <f>C5/B5-1</f>
-        <v>0.17956070629670173</v>
+        <v>6.8820295556564215E-2</v>
       </c>
       <c r="D6" s="10">
         <f>D5/C5-1</f>
-        <v>6.8820295556564215E-2</v>
+        <v>0.1566996201307127</v>
       </c>
       <c r="E6" s="10">
         <f>E5/D5-1</f>
-        <v>0.1566996201307127</v>
+        <v>0.14932156232406713</v>
       </c>
       <c r="F6" s="10">
         <f>F5/E5-1</f>
-        <v>0.14932156232406713</v>
+        <v>0.17788686799846665</v>
       </c>
       <c r="G6" s="10">
         <f>Assumptions!$B$5</f>
-        <v>0.16700000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="H6" s="10">
         <f>Assumptions!$B$6</f>
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="I6" s="10">
         <f>Assumptions!$B$7</f>
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="J6" s="10">
         <f>Assumptions!$B$8</f>
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="K6" s="10">
         <f>Assumptions!$B$9</f>
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B7" s="10">
-        <f>Historicals!C5</f>
-        <v>115856000000</v>
-      </c>
-      <c r="C7" s="10">
         <f>Historicals!C6</f>
         <v>135620000000</v>
       </c>
-      <c r="D7" s="10">
+      <c r="C7" s="10">
         <f>Historicals!C7</f>
         <v>146052000000</v>
       </c>
-      <c r="E7" s="10">
+      <c r="D7" s="10">
         <f>Historicals!C8</f>
         <v>171008000000</v>
       </c>
-      <c r="F7" s="10">
+      <c r="E7" s="10">
         <f>Historicals!C9</f>
         <v>193893000000</v>
       </c>
+      <c r="F7" s="10">
+        <f>Historicals!C10</f>
+        <v>225465000000</v>
+      </c>
       <c r="G7" s="10">
         <f>G5*Assumptions!$B$12</f>
-        <v>226273131000</v>
+        <v>263794050000.00003</v>
       </c>
       <c r="H7" s="10">
         <f>H5*Assumptions!$B$12</f>
-        <v>264739563270.00003</v>
+        <v>303363157500</v>
       </c>
       <c r="I7" s="10">
         <f>I5*Assumptions!$B$12</f>
-        <v>304450497760.5</v>
+        <v>342800367974.99994</v>
       </c>
       <c r="J7" s="10">
         <f>J5*Assumptions!$B$12</f>
-        <v>344029062469.36493</v>
+        <v>383936412132</v>
       </c>
       <c r="K7" s="10">
         <f>K5*Assumptions!$B$12</f>
-        <v>385312549965.68878</v>
+        <v>426169417466.52008</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B8" s="10">
         <f t="shared" ref="B8:K8" si="0">B7/B5</f>
-        <v>0.68925800771024703</v>
+        <v>0.68401674484289099</v>
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68401674484289099</v>
+        <v>0.68920085883491022</v>
       </c>
       <c r="D8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68920085883491022</v>
+        <v>0.69764443827971379</v>
       </c>
       <c r="E8" s="10">
         <f t="shared" si="0"/>
-        <v>0.69764443827971379</v>
+        <v>0.68823742386165188</v>
       </c>
       <c r="F8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
       <c r="G8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
       <c r="H8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
       <c r="I8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
       <c r="K8" s="10">
         <f t="shared" si="0"/>
-        <v>0.68823742386165188</v>
+        <v>0.67944093370580316</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B9" s="10">
-        <f>Historicals!D5</f>
-        <v>69916000000</v>
-      </c>
-      <c r="C9" s="10">
         <f>Historicals!D6</f>
         <v>83383000000</v>
       </c>
-      <c r="D9" s="10">
+      <c r="C9" s="10">
         <f>Historicals!D7</f>
         <v>88523000000</v>
       </c>
-      <c r="E9" s="10">
+      <c r="D9" s="10">
         <f>Historicals!D8</f>
         <v>109433000000</v>
       </c>
-      <c r="F9" s="10">
+      <c r="E9" s="10">
         <f>Historicals!D9</f>
         <v>128528000000</v>
       </c>
+      <c r="F9" s="10">
+        <f>Historicals!D10</f>
+        <v>155237000000</v>
+      </c>
       <c r="G9" s="10">
         <f>G5*Assumptions!$B$13</f>
-        <v>149992176000</v>
+        <v>181627290000</v>
       </c>
       <c r="H9" s="10">
         <f>H5*Assumptions!$B$13</f>
-        <v>175490845920</v>
+        <v>208871383499.99997</v>
       </c>
       <c r="I9" s="10">
         <f>I5*Assumptions!$B$13</f>
-        <v>201814472807.99997</v>
+        <v>236024663354.99994</v>
       </c>
       <c r="J9" s="10">
         <f>J5*Assumptions!$B$13</f>
-        <v>228050354273.03995</v>
+        <v>264347622957.59998</v>
       </c>
       <c r="K9" s="10">
         <f>K5*Assumptions!$B$13</f>
-        <v>255416396785.80478</v>
+        <v>293425861482.93604</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B10" s="10">
         <f t="shared" ref="B10:K10" si="1">B9/B5</f>
-        <v>0.41594878872971303</v>
+        <v>0.4205527815604983</v>
       </c>
       <c r="C10" s="10">
         <f t="shared" si="1"/>
-        <v>0.4205527815604983</v>
+        <v>0.41772880636104098</v>
       </c>
       <c r="D10" s="10">
         <f t="shared" si="1"/>
-        <v>0.41772880636104098</v>
+        <v>0.44644299573273716</v>
       </c>
       <c r="E10" s="10">
         <f t="shared" si="1"/>
-        <v>0.44644299573273716</v>
+        <v>0.45621956240859851</v>
       </c>
       <c r="F10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859851</v>
+        <v>0.46780818408927222</v>
       </c>
       <c r="G10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859851</v>
+        <v>0.46780818408927222</v>
       </c>
       <c r="H10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859851</v>
+        <v>0.46780818408927222</v>
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859846</v>
+        <v>0.46780818408927222</v>
       </c>
       <c r="J10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859851</v>
+        <v>0.46780818408927222</v>
       </c>
       <c r="K10" s="10">
         <f t="shared" si="1"/>
-        <v>0.45621956240859851</v>
+        <v>0.46780818408927222</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>71</v>
+        <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>101</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="G12" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="H12" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="I12" t="s">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="J12" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="K12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="16" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="B13" s="17">
-        <f>B9*(1-Historicals!H5)</f>
-        <v>60248983657.28109</v>
+        <f>B9*(1-Historicals!H6)</f>
+        <v>72448667566.53447</v>
       </c>
       <c r="C13" s="17">
-        <f>C9*(1-Historicals!H6)</f>
-        <v>72448667566.53447</v>
+        <f>C9*(1-Historicals!H7)</f>
+        <v>71722551566.996216</v>
       </c>
       <c r="D13" s="17">
-        <f>D9*(1-Historicals!H7)</f>
-        <v>71722551566.996231</v>
+        <f>D9*(1-Historicals!H8)</f>
+        <v>89481912364.199753</v>
       </c>
       <c r="E13" s="17">
-        <f>E9*(1-Historicals!H8)</f>
-        <v>89481912364.199768</v>
+        <f>E9*(1-Historicals!H9)</f>
+        <v>105868971147.07953</v>
       </c>
       <c r="F13" s="17">
-        <f>F9*(1-Historicals!H9)</f>
-        <v>105868971147.07953</v>
+        <f>F9*(1-Historicals!H10)</f>
+        <v>125126818572.44447</v>
       </c>
       <c r="G13" s="17">
         <f>G9*(1-Assumptions!$B$14)</f>
-        <v>123549089328.6418</v>
+        <v>146398377729.76004</v>
       </c>
       <c r="H13" s="17">
         <f>H9*(1-Assumptions!$B$14)</f>
-        <v>144552434514.51093</v>
+        <v>168358134389.22403</v>
       </c>
       <c r="I13" s="17">
         <f>I9*(1-Assumptions!$B$14)</f>
-        <v>166235299691.68753</v>
+        <v>190244691859.82312</v>
       </c>
       <c r="J13" s="17">
         <f>J9*(1-Assumptions!$B$14)</f>
-        <v>187845888651.6069</v>
+        <v>213074054883.00192</v>
       </c>
       <c r="K13" s="17">
         <f>K9*(1-Assumptions!$B$14)</f>
-        <v>210387395289.79974</v>
+        <v>236512200920.1322</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="B14" s="4">
-        <f>Historicals!I5</f>
-        <v>11689000000</v>
-      </c>
-      <c r="C14" s="4">
         <f>Historicals!I6</f>
         <v>14460000000</v>
       </c>
-      <c r="D14" s="4">
+      <c r="C14" s="4">
         <f>Historicals!I7</f>
         <v>13861000000</v>
       </c>
+      <c r="D14" s="4">
+        <f>Historicals!I8</f>
+        <v>20958000000</v>
+      </c>
       <c r="E14" s="4">
-        <f>Historicals!I8</f>
-        <v>22287000000</v>
+        <f>Historicals!I9</f>
+        <v>29433000000</v>
       </c>
       <c r="F14" s="4">
-        <f>Historicals!I9</f>
-        <v>34153000000</v>
+        <f>Historicals!I10</f>
+        <v>38534000000</v>
       </c>
       <c r="G14" s="4">
         <f>G5*Assumptions!$B$17</f>
-        <v>30417861888.78944</v>
+        <v>39614278117.433121</v>
       </c>
       <c r="H14" s="4">
         <f>H5*Assumptions!$B$17</f>
-        <v>35588898409.883644</v>
+        <v>45556419835.048088</v>
       </c>
       <c r="I14" s="4">
         <f>I5*Assumptions!$B$17</f>
-        <v>40927233171.366188</v>
+        <v>51478754413.604332</v>
       </c>
       <c r="J14" s="4">
         <f>J5*Assumptions!$B$17</f>
-        <v>46247773483.643784</v>
+        <v>57656204943.236862</v>
       </c>
       <c r="K14" s="4">
         <f>K5*Assumptions!$B$17</f>
-        <v>51797506301.681046</v>
+        <v>63998387486.99292</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="B15" s="4">
-        <f>Historicals!J5</f>
-        <v>20622000000</v>
-      </c>
-      <c r="C15" s="4">
         <f>Historicals!J6</f>
         <v>23886000000</v>
       </c>
-      <c r="D15" s="4">
+      <c r="C15" s="4">
         <f>Historicals!J7</f>
         <v>28107000000</v>
       </c>
-      <c r="E15" s="4">
+      <c r="D15" s="4">
         <f>Historicals!J8</f>
         <v>44477000000</v>
       </c>
-      <c r="F15" s="4">
+      <c r="E15" s="4">
         <f>Historicals!J9</f>
         <v>64551000000</v>
       </c>
+      <c r="F15" s="4">
+        <f>Historicals!J10</f>
+        <v>115948000000</v>
+      </c>
       <c r="G15" s="10">
         <f>G5*Assumptions!$B$18</f>
-        <v>98631572400</v>
+        <v>116475489000</v>
       </c>
       <c r="H15" s="10">
         <f>H5*Assumptions!$C$18</f>
-        <v>92319151766.399994</v>
+        <v>107157449879.99998</v>
       </c>
       <c r="I15" s="10">
         <f>I5*Assumptions!$D$18</f>
-        <v>79625268398.519989</v>
+        <v>90815938773.299973</v>
       </c>
       <c r="J15" s="10">
         <f>J5*Assumptions!$E$18</f>
-        <v>69981763670.254791</v>
+        <v>79110773331.408005</v>
       </c>
       <c r="K15" s="10">
         <f>K5*Assumptions!$F$18</f>
-        <v>61583952029.824219</v>
+        <v>68995895884.035126</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="B16" s="10">
-        <v>-2700000000</v>
-      </c>
-      <c r="C16" s="10">
         <f>Historicals!N6-Historicals!N5</f>
         <v>-21147000000</v>
       </c>
-      <c r="D16" s="10">
+      <c r="C16" s="10">
         <f>Historicals!N7-Historicals!N6</f>
         <v>5506000000</v>
       </c>
-      <c r="E16" s="10">
+      <c r="D16" s="10">
         <f>Historicals!N8-Historicals!N7</f>
         <v>-45660000000</v>
       </c>
-      <c r="F16" s="10">
+      <c r="E16" s="10">
         <f>Historicals!N9-Historicals!N8</f>
         <v>15465000000</v>
       </c>
+      <c r="F16" s="10">
+        <f>Historicals!N10-Historicals!N9</f>
+        <v>-11028000000</v>
+      </c>
       <c r="G16" s="10">
         <f>(G5-F5)*Assumptions!$B$19</f>
-        <v>1411437240</v>
+        <v>1692378900</v>
       </c>
       <c r="H16" s="10">
         <f>(H5-G5)*Assumptions!$B$19</f>
-        <v>1676736730.8</v>
+        <v>1747132334.9999981</v>
       </c>
       <c r="I16" s="10">
         <f>(I5-H5)*Assumptions!$B$19</f>
-        <v>1730984095.6199982</v>
+        <v>1741308560.549998</v>
       </c>
       <c r="J16" s="10">
         <f>(J5-I5)*Assumptions!$B$19</f>
-        <v>1725214148.6345983</v>
+        <v>1816318775.4660022</v>
       </c>
       <c r="K16" s="10">
         <f>(K5-J5)*Assumptions!$B$19</f>
-        <v>1799531065.8065534</v>
+        <v>1864753942.8117626</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="B18" s="4">
         <f t="shared" ref="B18:K18" si="2">B13 + B14 - B15 - B16</f>
-        <v>54015983657.281097</v>
+        <v>84169667566.53447</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="2"/>
-        <v>84169667566.53447</v>
+        <v>51970551566.996216</v>
       </c>
       <c r="D18" s="4">
         <f t="shared" si="2"/>
-        <v>51970551566.996231</v>
+        <v>111622912364.19975</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="2"/>
-        <v>112951912364.19977</v>
+        <v>55285971147.079529</v>
       </c>
       <c r="F18" s="4">
         <f t="shared" si="2"/>
-        <v>60005971147.079529</v>
+        <v>58740818572.444458</v>
       </c>
       <c r="G18" s="4">
         <f t="shared" si="2"/>
-        <v>53923941577.431244</v>
+        <v>67844787947.193176</v>
       </c>
       <c r="H18" s="4">
         <f t="shared" si="2"/>
-        <v>86145444427.194565</v>
+        <v>105009972009.27214</v>
       </c>
       <c r="I18" s="4">
         <f t="shared" si="2"/>
-        <v>125806280368.91373</v>
+        <v>149166198939.57751</v>
       </c>
       <c r="J18" s="4">
         <f t="shared" si="2"/>
-        <v>162386684316.36127</v>
+        <v>189803167719.36475</v>
       </c>
       <c r="K18" s="4">
         <f t="shared" si="2"/>
-        <v>198801418495.85001</v>
+        <v>229649938580.27823</v>
       </c>
     </row>
   </sheetData>
@@ -2414,129 +2534,134 @@
     <col min="6" max="6" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>29</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>119</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="10">
-        <v>1</v>
-      </c>
-      <c r="C6" s="10">
-        <v>2</v>
-      </c>
-      <c r="D6" s="10">
-        <v>3</v>
-      </c>
-      <c r="E6" s="10">
-        <v>4</v>
-      </c>
-      <c r="F6" s="10">
-        <v>5</v>
+        <v>120</v>
+      </c>
+      <c r="B6" s="27">
+        <f>Assumptions!$B$42</f>
+        <v>0.67671232876712328</v>
+      </c>
+      <c r="C6" s="27">
+        <f>B6+1</f>
+        <v>1.6767123287671233</v>
+      </c>
+      <c r="D6" s="27">
+        <f>C6+1</f>
+        <v>2.6767123287671231</v>
+      </c>
+      <c r="E6" s="27">
+        <f>D6+1</f>
+        <v>3.6767123287671231</v>
+      </c>
+      <c r="F6" s="27">
+        <f>E6+1</f>
+        <v>4.6767123287671231</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="B7" s="10">
-        <f>Forecast!G18</f>
-        <v>53923941577.431244</v>
+        <f>Forecast!G18*Assumptions!$B$42</f>
+        <v>45911404446.456749</v>
       </c>
       <c r="C7" s="10">
         <f>Forecast!H18</f>
-        <v>86145444427.194565</v>
+        <v>105009972009.27214</v>
       </c>
       <c r="D7" s="10">
         <f>Forecast!I18</f>
-        <v>125806280368.91373</v>
+        <v>149166198939.57751</v>
       </c>
       <c r="E7" s="10">
         <f>Forecast!J18</f>
-        <v>162386684316.36127</v>
+        <v>189803167719.36475</v>
       </c>
       <c r="F7" s="10">
         <f>Forecast!K18</f>
-        <v>198801418495.85001</v>
+        <v>229649938580.27823</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>122</v>
       </c>
       <c r="B8" s="10">
-        <f>1/(1+Assumptions!B30)^B6</f>
-        <v>0.91914383869720317</v>
+        <f>1/(1+Assumptions!$B$30)^B6</f>
+        <v>0.94050286029824959</v>
       </c>
       <c r="C8" s="10">
         <f>1/(1+Assumptions!$B$30)^C6</f>
-        <v>0.84482539621503028</v>
+        <v>0.85900065977774087</v>
       </c>
       <c r="D8" s="10">
         <f>1/(1+Assumptions!$B$30)^D6</f>
-        <v>0.77651605770596854</v>
+        <v>0.78456128593229291</v>
       </c>
       <c r="E8" s="10">
         <f>1/(1+Assumptions!$B$30)^E6</f>
-        <v>0.71372995008988283</v>
+        <v>0.71657268754950409</v>
       </c>
       <c r="F8" s="10">
         <f>1/(1+Assumptions!$B$30)^F6</f>
-        <v>0.65602048611877817</v>
+        <v>0.6544758526183917</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="B9" s="10">
         <f>B7*B8</f>
-        <v>49563858659.163872</v>
+        <v>43179807202.202347</v>
       </c>
       <c r="C9" s="10">
         <f>C7*C8</f>
-        <v>72777859220.324524</v>
+        <v>90203635239.206863</v>
       </c>
       <c r="D9" s="10">
         <f>D7*D8</f>
-        <v>97690596866.720673</v>
+        <v>117030024857.66716</v>
       </c>
       <c r="E9" s="10">
         <f>E7*E8</f>
-        <v>115900240092.37808</v>
+        <v>136007765998.07448</v>
       </c>
       <c r="F9" s="10">
         <f>F7*F8</f>
-        <v>130417803202.75018</v>
+        <v>150300339356.08887</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2548,11 +2673,11 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>89</v>
+        <v>124</v>
       </c>
       <c r="B11" s="10">
         <f>SUM(B9:F9)</f>
-        <v>466350358041.33734</v>
+        <v>536721572653.23969</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -2568,11 +2693,11 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="B13" s="10">
         <f>Forecast!K18*(1+Assumptions!$B$33)</f>
-        <v>204765461050.72552</v>
+        <v>236539436737.68658</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -2581,11 +2706,11 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>126</v>
       </c>
       <c r="B14" s="10">
-        <f>B13*(1+Assumptions!B33)/(Assumptions!B30-Assumptions!B33)</f>
-        <v>3638296967857.4033</v>
+        <f>B13/(Assumptions!B30-Assumptions!B33)</f>
+        <v>3645784707685.9346</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -2594,11 +2719,11 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>127</v>
       </c>
       <c r="B15" s="10">
-        <f>B14/(1+Assumptions!$B$30)^5</f>
-        <v>2386797345498.29</v>
+        <f>B14/(1+Assumptions!$B$30)^F6</f>
+        <v>2386078055025.8462</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -2614,11 +2739,11 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="B17" s="10">
         <f>B11+B15</f>
-        <v>2853147703539.6274</v>
+        <v>2922799627679.0859</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -2642,11 +2767,11 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>85</v>
+        <v>129</v>
       </c>
       <c r="B20" s="10">
-        <f>[0]!latest_debt_cell</f>
-        <v>60588000000</v>
+        <f>Historicals!L10</f>
+        <v>56826000000</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -2655,11 +2780,11 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>130</v>
       </c>
       <c r="B21" s="10">
-        <f>[0]!latest_cash_cell</f>
-        <v>30242000000</v>
+        <f>Historicals!O10</f>
+        <v>76651000000</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -2668,11 +2793,11 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>131</v>
       </c>
       <c r="B22" s="10">
         <f>B17-B20+B21</f>
-        <v>2822801703539.6274</v>
+        <v>2942624627679.0859</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -2689,11 +2814,11 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B24" s="10">
         <f>Assumptions!$B$36</f>
-        <v>7425629076</v>
+        <v>7425545491</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -2702,11 +2827,11 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>132</v>
       </c>
       <c r="B25" s="10">
         <f>B22/B24</f>
-        <v>380.14310634812909</v>
+        <v>396.28396745338665</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -2715,11 +2840,11 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="B26" s="10">
         <f>Assumptions!$B$37</f>
-        <v>424.16</v>
+        <v>532.6</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -2728,11 +2853,11 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>91</v>
+        <v>133</v>
       </c>
       <c r="B27" s="14">
         <f>(B25-B26)/B26</f>
-        <v>-0.10377426832296993</v>
+        <v>-0.25594448469135067</v>
       </c>
     </row>
   </sheetData>
@@ -2748,21 +2873,21 @@
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>30</v>
+        <v>134</v>
       </c>
       <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="B3" s="22"/>
       <c r="C3" s="23"/>
@@ -2772,8 +2897,9 @@
       <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="21" t="s">
-        <v>113</v>
+      <c r="A4" s="21" t="str">
+        <f>"WACC vs. Terminal Growth Rate | Base Case: "&amp;TEXT(DCF!B25,"$0.00")&amp;" | Current Price: "&amp;TEXT(Assumptions!B37,"$0.00")</f>
+        <v>WACC vs. Terminal Growth Rate | Base Case: $396.28 | Current Price: $532.60</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="23"/>
@@ -2782,16 +2908,16 @@
       <c r="F4" s="23"/>
       <c r="G4" s="23"/>
     </row>
-    <row r="7" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D7" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="10">
         <f>DCF!B25</f>
-        <v>380.14310634812909</v>
+        <v>396.28396745338665</v>
       </c>
       <c r="C8" s="5">
         <v>0.02</v>
@@ -2811,126 +2937,156 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B9" s="5">
-        <v>7.4999999999999997E-2</v>
+        <v>0.08</v>
       </c>
       <c r="C9">
-        <v>414.13054049429786</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B9-C$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>444.99446041993963</v>
       </c>
       <c r="D9">
-        <v>453.22033957120163</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B9-D$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>480.30501195840935</v>
       </c>
       <c r="E9">
-        <v>501.01748122080363</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B9-E$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>522.67767380457303</v>
       </c>
       <c r="F9">
-        <v>560.78721890786539</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B9-F$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>574.46648272766197</v>
       </c>
       <c r="G9">
-        <v>637.66066521987</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B9-G$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>639.2024938815232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
-        <v>0.08</v>
+        <v>8.5000000000000006E-2</v>
       </c>
       <c r="C10">
-        <v>376.27601917938779</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B10-C$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>408.43939669658744</v>
       </c>
       <c r="D10">
-        <v>408.38603873085748</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B10-D$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>437.81443304551175</v>
       </c>
       <c r="E10">
-        <v>446.93628299298564</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B10-E$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>472.53038509424067</v>
       </c>
       <c r="F10">
-        <v>494.07349353599176</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B10-F$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>514.18952755271528</v>
       </c>
       <c r="G10">
-        <v>553.01778271520504</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B10-G$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>565.10625722418433</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="24">
-        <v>8.5000000000000006E-2</v>
+        <v>0.09</v>
       </c>
       <c r="C11">
-        <v>344.29623880835265</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B11-C$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>377.14627654098115</v>
       </c>
       <c r="D11">
-        <v>371.07936440594028</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B11-D$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>401.90282592952701</v>
       </c>
       <c r="E11">
-        <v>402.74833540118306</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B11-E$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>430.78546688283075</v>
       </c>
       <c r="F11">
-        <v>440.76890541337741</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B11-F$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>464.9194971003713</v>
       </c>
       <c r="G11">
-        <v>487.25827411484067</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B11-G$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>505.88033336142013</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B12" s="5">
-        <v>0.09</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="C12">
-        <v>316.93118254611159</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B12-C$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>350.06188705886723</v>
       </c>
       <c r="D12">
-        <v>339.5619329607203</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B12-D$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>371.15954727374213</v>
       </c>
       <c r="E12">
-        <v>365.97897526098347</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B12-E$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>395.50300136782863</v>
       </c>
       <c r="F12">
-        <v>397.21493450662462</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B12-F$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>423.90369781092937</v>
       </c>
       <c r="G12">
-        <v>434.7154857812576</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B12-G$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>457.46815724368497</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B13" s="5">
-        <v>9.5000000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="C13">
-        <v>293.25686946679474</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B13-C$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>326.39633967811307</v>
       </c>
       <c r="D13">
-        <v>312.59207584540542</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B13-D$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>344.55014729191748</v>
       </c>
       <c r="E13">
-        <v>334.91501130298684</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B13-E$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>365.29735599340847</v>
       </c>
       <c r="F13">
-        <v>360.97260810928162</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B13-F$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>389.23644295666719</v>
       </c>
       <c r="G13">
-        <v>391.78341026848449</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B13-G$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>417.16537774713578</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="14"/>
       <c r="B14" s="5">
-        <v>0.1</v>
+        <v>0.105</v>
       </c>
       <c r="C14">
-        <v>272.58034231860574</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B14-C$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>305.54562118001093</v>
       </c>
       <c r="D14">
-        <v>289.2592668016643</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B14-D$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>321.29880860096449</v>
       </c>
       <c r="E14">
-        <v>308.33276871999828</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B14-E$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>339.15242101137852</v>
       </c>
       <c r="F14">
-        <v>330.35344286636354</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B14-F$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>359.55654948042314</v>
       </c>
       <c r="G14">
-        <v>356.05808229776778</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B14-G$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
+        <v>383.09977463701307</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -2940,24 +3096,75 @@
       <c r="A16" s="14"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C9:G14">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="lessThan">
-      <formula>424.16</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
-      <formula>424.16</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
-      <formula>424.16</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="greaterThan">
-      <formula>424.16</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="greaterThan">
-      <formula>424.16</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="1" operator="lessThan" id="{00000000-000E-0000-0500-000001000000}">
+            <xm:f>Assumptions!$B$37</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="2" operator="greaterThan" id="{00000000-000E-0000-0500-000002000000}">
+            <xm:f>Assumptions!$B$37</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="3" operator="greaterThan" id="{00000000-000E-0000-0500-000003000000}">
+            <xm:f>Assumptions!$B$37</xm:f>
+            <x14:dxf>
+              <font>
+                <color theme="0"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="4" operator="greaterThan" id="{00000000-000E-0000-0500-000004000000}">
+            <xm:f>Assumptions!$B$37</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00B050"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="5" operator="greaterThan" id="{00000000-000E-0000-0500-000005000000}">
+            <xm:f>Assumptions!$B$37</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>C9:G14</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2966,109 +3173,123 @@
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="str">
+        <f>"Valuation date: "&amp;TEXT(Assumptions!B40,"mm/dd/yyyy")</f>
+        <v>Valuation date: 10/26/2026</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>116</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>117</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>118</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>119</v>
+      <c r="A7" t="str">
+        <f>"Market Cap | "&amp;TEXT(Profile!B7/1000000000000,"$0.00")&amp;"T"</f>
+        <v>Market Cap | $3.95T</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>120</v>
+      <c r="A8" t="str">
+        <f>"Current Price | "&amp;TEXT(Assumptions!B37,"$0.00")</f>
+        <v>Current Price | $532.60</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>126</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>121</v>
+      <c r="A11" t="str">
+        <f>"Intrinsic Value Per Share | "&amp;TEXT(DCF!B25,"$0.00")</f>
+        <v>Intrinsic Value Per Share | $396.28</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>122</v>
+      <c r="A12" t="str">
+        <f>"Current Market Price | "&amp;TEXT(Assumptions!B37,"$0.00")</f>
+        <v>Current Market Price | $532.60</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>123</v>
+      <c r="A13" t="str">
+        <f>"Implied Upside / Downside | "&amp;TEXT(DCF!B27,"0.00%")</f>
+        <v>Implied Upside / Downside | -25.59%</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>125</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>127</v>
+      <c r="A17" t="str">
+        <f>"WACC | "&amp;TEXT(Assumptions!B30,"0.00%")</f>
+        <v>WACC | 9.49%</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>128</v>
+      <c r="A18" t="str">
+        <f>"Terminal Growth Rate | "&amp;TEXT(Assumptions!B33,"0.00%")</f>
+        <v>Terminal Growth Rate | 3.00%</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>130</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>129</v>
+      <c r="A20" t="str">
+        <f>"FY2031E Revenue | "&amp;TEXT(Forecast!K5/1000000000,"$#,##0.0")&amp;"B"</f>
+        <v>FY2031E Revenue | $627.2B</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>131</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>132</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>133</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>134</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Take the EV bridge from the FY2026 10-K
Count all $66.6B of finance lease liabilities as debt (Yahoo's total debt
had $16.5B), add long-term equity investments at carrying value, use
diluted shares, and set the cost of debt above the risk-free rate. Value
moves from $396.28 to $395.95. Restore the sensitivity grid's conditional
formatting and list the open judgment calls in the README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/MSFT_DCF_Model.xlsx
+++ b/excel/MSFT_DCF_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/masontrinkner/ClaudeCode/msft-dcf-valuation/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEC767A-91AB-A347-BC7D-97B233354D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{764E031C-4C50-6F4C-B200-0429BCB610A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17420" yWindow="780" windowWidth="16780" windowHeight="21460" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="153">
   <si>
     <t>MSFT DCF Model - Summary</t>
   </si>
@@ -242,7 +242,7 @@
     <t>Change NWC as % of Rev Change</t>
   </si>
   <si>
-    <t>3yr avg FY2023-FY2025</t>
+    <t>Assumption. Historical NWC changes swing from -$46B to +$16B because current assets include cash and investments, so they don't give a usable average</t>
   </si>
   <si>
     <t>WACC INPUTS</t>
@@ -272,7 +272,7 @@
     <t>Pre-tax Cost of Debt</t>
   </si>
   <si>
-    <t>Aprox MSFT bond yield, Alpha Spread</t>
+    <t>10Y Treasury + ~40bp (AAA-rated; approx.). Was 3.5%, below the risk-free rate</t>
   </si>
   <si>
     <t>After-tax Cost of Debt</t>
@@ -284,7 +284,7 @@
     <t>Debt Weight</t>
   </si>
   <si>
-    <t>Market value: total debt / (total debt + market cap)</t>
+    <t>Market value: debt incl. finance leases / (debt + market cap)</t>
   </si>
   <si>
     <t>Equity Rate</t>
@@ -311,7 +311,10 @@
     <t>SHARES &amp; PRICE</t>
   </si>
   <si>
-    <t>yfinance</t>
+    <t>Diluted Shares Outstanding</t>
+  </si>
+  <si>
+    <t>Basic shares (Yahoo, 10/26/26) + FY2026 dilution</t>
   </si>
   <si>
     <t>Current Stock Price</t>
@@ -341,6 +344,45 @@
     <t>Share of FY2027E cash flow still ahead of the valuation date</t>
   </si>
   <si>
+    <t>BALANCE SHEET (FY2026 10-K, 6/30/2026)</t>
+  </si>
+  <si>
+    <t>Long-Term Debt (incl. current portion)</t>
+  </si>
+  <si>
+    <t>10-K: LongTermDebt</t>
+  </si>
+  <si>
+    <t>Finance Lease Liabilities</t>
+  </si>
+  <si>
+    <t>10-K lease note; Yahoo 'Total Debt' only includes $16.5B of this</t>
+  </si>
+  <si>
+    <t>Total Debt incl. Finance Leases</t>
+  </si>
+  <si>
+    <t>Operating leases excluded (their cost is in EBIT)</t>
+  </si>
+  <si>
+    <t>Cash &amp; Short-Term Investments</t>
+  </si>
+  <si>
+    <t>10-K balance sheet</t>
+  </si>
+  <si>
+    <t>Long-Term Equity Investments</t>
+  </si>
+  <si>
+    <t>10-K carrying value (incl. OpenAI stake); market value is likely far higher</t>
+  </si>
+  <si>
+    <t>Dilutive Securities (shares)</t>
+  </si>
+  <si>
+    <t>FY2026 diluted minus basic weighted shares (10-K)</t>
+  </si>
+  <si>
     <t>MSFT DCF Model - Forecast</t>
   </si>
   <si>
@@ -428,10 +470,13 @@
     <t>Enterprise Value</t>
   </si>
   <si>
-    <t>Less: Total Debt</t>
+    <t>Less: Total Debt incl. Finance Leases</t>
   </si>
   <si>
     <t>Plus: Cash &amp; Short-Term Investments</t>
+  </si>
+  <si>
+    <t>Plus: Long-Term Equity Investments</t>
   </si>
   <si>
     <t>Equity Value</t>
@@ -463,7 +508,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00,,,&quot;T&quot;"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -626,7 +671,7 @@
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -635,47 +680,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -1509,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.6640625" customWidth="1"/>
@@ -1756,7 +1774,8 @@
         <v>76</v>
       </c>
       <c r="B26" s="15">
-        <v>3.5000000000000003E-2</v>
+        <f>B22+0.004</f>
+        <v>5.3900000000000003E-2</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>77</v>
@@ -1768,7 +1787,7 @@
       </c>
       <c r="B27" s="14">
         <f>B26*(1-B14)</f>
-        <v>2.8211306905155067E-2</v>
+        <v>4.34454126339388E-2</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>79</v>
@@ -1779,8 +1798,8 @@
         <v>80</v>
       </c>
       <c r="B28" s="15">
-        <f>Historicals!L10/(Historicals!L10+Profile!B7)</f>
-        <v>1.4165168102379019E-2</v>
+        <f>B47/(B47+Profile!B7)</f>
+        <v>2.6315858037410659E-2</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>81</v>
@@ -1792,7 +1811,7 @@
       </c>
       <c r="B29" s="14">
         <f>1-B28</f>
-        <v>0.985834831897621</v>
+        <v>0.97368414196258934</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>83</v>
@@ -1804,7 +1823,7 @@
       </c>
       <c r="B30" s="14">
         <f>B29*B25+B28*B27</f>
-        <v>9.4880253691069907E-2</v>
+        <v>9.445943884549049E-2</v>
       </c>
       <c r="C30" s="18" t="s">
         <v>85</v>
@@ -1837,65 +1856,65 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="B36">
-        <f>Profile!B6</f>
-        <v>7425545491</v>
+        <f>Profile!B6+B50</f>
+        <v>7449545491</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B37">
         <f>Profile!B8</f>
         <v>532.6</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B40" s="25">
         <v>46321</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B41" s="25">
         <v>46568</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" s="26">
         <f>(B41-B40)/365</f>
         <v>0.67671232876712328</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
@@ -1907,19 +1926,78 @@
       <c r="C43" s="5"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="9" t="s">
+        <v>101</v>
+      </c>
       <c r="C44" s="5"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C45" s="5"/>
+      <c r="A45" t="s">
+        <v>102</v>
+      </c>
+      <c r="B45" s="4">
+        <v>40294000000</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C46" s="5"/>
+      <c r="A46" t="s">
+        <v>104</v>
+      </c>
+      <c r="B46" s="4">
+        <v>66594000000</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C47" s="5"/>
+      <c r="A47" t="s">
+        <v>106</v>
+      </c>
+      <c r="B47" s="4">
+        <f>B45+B46</f>
+        <v>106888000000</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C48" s="5"/>
+      <c r="A48" t="s">
+        <v>108</v>
+      </c>
+      <c r="B48" s="4">
+        <v>76843000000</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>110</v>
+      </c>
+      <c r="B49" s="4">
+        <v>36348000000</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>112</v>
+      </c>
+      <c r="B50" s="4">
+        <f>7453000000-7429000000</f>
+        <v>24000000</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>113</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1946,7 +2024,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -1956,34 +2034,34 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="E4" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="F4" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="G4" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="H4" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="I4" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="J4" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="K4" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
@@ -2033,7 +2111,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B6" s="10">
         <f>B5/Historicals!B5-1</f>
@@ -2258,42 +2336,42 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="C12" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="F12" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="G12" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="I12" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="J12" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="K12" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B13" s="17">
         <f>B9*(1-Historicals!H6)</f>
@@ -2338,7 +2416,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B14" s="4">
         <f>Historicals!I6</f>
@@ -2383,7 +2461,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B15" s="4">
         <f>Historicals!J6</f>
@@ -2428,7 +2506,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B16" s="10">
         <f>Historicals!N6-Historicals!N5</f>
@@ -2473,7 +2551,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B18" s="4">
         <f t="shared" ref="B18:K18" si="2">B13 + B14 - B15 - B16</f>
@@ -2536,7 +2614,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -2546,27 +2624,27 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B6" s="27">
         <f>Assumptions!$B$42</f>
@@ -2591,7 +2669,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B7" s="10">
         <f>Forecast!G18*Assumptions!$B$42</f>
@@ -2616,52 +2694,52 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B8" s="10">
         <f>1/(1+Assumptions!$B$30)^B6</f>
-        <v>0.94050286029824959</v>
+        <v>0.94074755727447745</v>
       </c>
       <c r="C8" s="10">
         <f>1/(1+Assumptions!$B$30)^C6</f>
-        <v>0.85900065977774087</v>
+        <v>0.85955451968767449</v>
       </c>
       <c r="D8" s="10">
         <f>1/(1+Assumptions!$B$30)^D6</f>
-        <v>0.78456128593229291</v>
+        <v>0.78536900425875122</v>
       </c>
       <c r="E8" s="10">
         <f>1/(1+Assumptions!$B$30)^E6</f>
-        <v>0.71657268754950409</v>
+        <v>0.71758621323345839</v>
       </c>
       <c r="F8" s="10">
         <f>1/(1+Assumptions!$B$30)^F6</f>
-        <v>0.6544758526183917</v>
+        <v>0.65565354709756685</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B9" s="10">
         <f>B7*B8</f>
-        <v>43179807202.202347</v>
+        <v>43191041584.044769</v>
       </c>
       <c r="C9" s="10">
         <f>C7*C8</f>
-        <v>90203635239.206863</v>
+        <v>90261796052.846054</v>
       </c>
       <c r="D9" s="10">
         <f>D7*D8</f>
-        <v>117030024857.66716</v>
+        <v>117150509130.23878</v>
       </c>
       <c r="E9" s="10">
         <f>E7*E8</f>
-        <v>136007765998.07448</v>
+        <v>136200136383.45393</v>
       </c>
       <c r="F9" s="10">
         <f>F7*F8</f>
-        <v>150300339356.08887</v>
+        <v>150570796820.8978</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -2673,11 +2751,11 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B11" s="10">
         <f>SUM(B9:F9)</f>
-        <v>536721572653.23969</v>
+        <v>537374279971.48132</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -2693,7 +2771,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B13" s="10">
         <f>Forecast!K18*(1+Assumptions!$B$33)</f>
@@ -2706,11 +2784,11 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B14" s="10">
         <f>B13/(Assumptions!B30-Assumptions!B33)</f>
-        <v>3645784707685.9346</v>
+        <v>3669585726687.3276</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -2719,11 +2797,11 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B15" s="10">
         <f>B14/(1+Assumptions!$B$30)^F6</f>
-        <v>2386078055025.8462</v>
+        <v>2405976898081.1489</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -2739,11 +2817,11 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B17" s="10">
         <f>B11+B15</f>
-        <v>2922799627679.0859</v>
+        <v>2943351178052.6304</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -2767,11 +2845,11 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B20" s="10">
-        <f>Historicals!L10</f>
-        <v>56826000000</v>
+        <f>Assumptions!B47</f>
+        <v>106888000000</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -2780,11 +2858,11 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B21" s="10">
-        <f>Historicals!O10</f>
-        <v>76651000000</v>
+        <f>Assumptions!B48</f>
+        <v>76843000000</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -2793,11 +2871,11 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B22" s="10">
-        <f>B17-B20+B21</f>
-        <v>2942624627679.0859</v>
+        <f>Assumptions!B49</f>
+        <v>36348000000</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -2805,8 +2883,13 @@
       <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
+      <c r="A23" t="s">
+        <v>146</v>
+      </c>
+      <c r="B23" s="10">
+        <f>B17-B20+B21+B22</f>
+        <v>2949654178052.6304</v>
+      </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -2814,11 +2897,11 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="B24" s="10">
         <f>Assumptions!$B$36</f>
-        <v>7425545491</v>
+        <v>7449545491</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -2827,11 +2910,11 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="B25" s="10">
-        <f>B22/B24</f>
-        <v>396.28396745338665</v>
+        <f>B23/B24</f>
+        <v>395.95089144917478</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -2840,7 +2923,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B26" s="10">
         <f>Assumptions!$B$37</f>
@@ -2853,11 +2936,11 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="B27" s="14">
         <f>(B25-B26)/B26</f>
-        <v>-0.25594448469135067</v>
+        <v>-0.25656986209317545</v>
       </c>
     </row>
   </sheetData>
@@ -2875,7 +2958,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="I1" s="14"/>
     </row>
@@ -2887,7 +2970,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="B3" s="22"/>
       <c r="C3" s="23"/>
@@ -2899,7 +2982,7 @@
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="str">
         <f>"WACC vs. Terminal Growth Rate | Base Case: "&amp;TEXT(DCF!B25,"$0.00")&amp;" | Current Price: "&amp;TEXT(Assumptions!B37,"$0.00")</f>
-        <v>WACC vs. Terminal Growth Rate | Base Case: $396.28 | Current Price: $532.60</v>
+        <v>WACC vs. Terminal Growth Rate | Base Case: $395.95 | Current Price: $532.60</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="23"/>
@@ -2910,14 +2993,14 @@
     </row>
     <row r="7" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D7" s="9" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="10">
         <f>DCF!B25</f>
-        <v>396.28396745338665</v>
+        <v>395.95089144917478</v>
       </c>
       <c r="C8" s="5">
         <v>0.02</v>
@@ -2937,30 +3020,30 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="B9" s="5">
         <v>0.08</v>
       </c>
       <c r="C9">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B9-C$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>444.99446041993963</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B9-C$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>441.74568946078278</v>
       </c>
       <c r="D9">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B9-D$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>480.30501195840935</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B9-D$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>476.9424819467107</v>
       </c>
       <c r="E9">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B9-E$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>522.67767380457303</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B9-E$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>519.17863292982418</v>
       </c>
       <c r="F9">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B9-F$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>574.46648272766197</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B9-F$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>570.80059524251851</v>
       </c>
       <c r="G9">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B9-G$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>639.2024938815232</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B9)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B9-G$8)/(1+$B9)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>635.32804813338635</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -2968,24 +3051,24 @@
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="C10">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B10-C$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>408.43939669658744</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B10-C$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>405.30839420134834</v>
       </c>
       <c r="D10">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B10-D$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>437.81443304551175</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B10-D$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>434.5887937871002</v>
       </c>
       <c r="E10">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B10-E$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>472.53038509424067</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B10-E$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>469.19290238844349</v>
       </c>
       <c r="F10">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B10-F$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>514.18952755271528</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B10-F$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>510.7178327100554</v>
       </c>
       <c r="G10">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B10-G$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>565.10625722418433</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B10)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B10-G$8)/(1+$B10)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>561.47052532535872</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -2993,24 +3076,24 @@
         <v>0.09</v>
       </c>
       <c r="C11">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B11-C$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>377.14627654098115</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B11-C$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>374.11609024783684</v>
       </c>
       <c r="D11">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B11-D$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>401.90282592952701</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B11-D$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>398.79288212821751</v>
       </c>
       <c r="E11">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B11-E$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>430.78546688283075</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B11-E$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>427.58247265532856</v>
       </c>
       <c r="F11">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B11-F$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>464.9194971003713</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B11-F$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>461.60653418736871</v>
       </c>
       <c r="G11">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B11-G$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>505.88033336142013</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B11)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B11-G$8)/(1+$B11)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>502.43540802581697</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -3018,24 +3101,24 @@
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="C12">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B12-C$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>350.06188705886723</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B12-C$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>347.11895781359999</v>
       </c>
       <c r="D12">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B12-D$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>371.15954727374213</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B12-D$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>368.14864826498143</v>
       </c>
       <c r="E12">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B12-E$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>395.50300136782863</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B12-E$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>392.41367570888315</v>
       </c>
       <c r="F12">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B12-F$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>423.90369781092937</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B12-F$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>420.72287439343506</v>
       </c>
       <c r="G12">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B12-G$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>457.46815724368497</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B12)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B12-G$8)/(1+$B12)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>454.17920011154195</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -3043,24 +3126,24 @@
         <v>0.1</v>
       </c>
       <c r="C13">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B13-C$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>326.39633967811307</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B13-C$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>323.5296530892366</v>
       </c>
       <c r="D13">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B13-D$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>344.55014729191748</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B13-D$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>341.62497507015809</v>
       </c>
       <c r="E13">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B13-E$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>365.29735599340847</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B13-E$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>362.3053430483543</v>
       </c>
       <c r="F13">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B13-F$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>389.23644295666719</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B13-F$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>386.16730610011905</v>
       </c>
       <c r="G13">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B13-G$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>417.16537774713578</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B13)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B13-G$8)/(1+$B13)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>414.00626299384464</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -3069,24 +3152,24 @@
         <v>0.105</v>
       </c>
       <c r="C14">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B14-C$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>305.54562118001093</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+C$8)/($B14-C$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>302.74610878915223</v>
       </c>
       <c r="D14">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B14-D$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>321.29880860096449</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+D$8)/($B14-D$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>318.44854459061975</v>
       </c>
       <c r="E14">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B14-E$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>339.15242101137852</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+E$8)/($B14-E$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>336.24463849894966</v>
       </c>
       <c r="F14">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B14-F$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>359.55654948042314</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+F$8)/($B14-F$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>356.58303153704099</v>
       </c>
       <c r="G14">
-        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B14-G$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21)/DCF!$B$24</f>
-        <v>383.09977463701307</v>
+        <f>(SUMPRODUCT(DCF!$B$7:$F$7/(1+$B14)^DCF!$B$6:$F$6)+DCF!$F$7*(1+G$8)/($B14-G$8)/(1+$B14)^DCF!$F$6-DCF!$B$20+DCF!$B$21+DCF!$B$22)/DCF!$B$24</f>
+        <v>380.05040811945406</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -3105,7 +3188,7 @@
             <xm:f>Assumptions!$B$37</xm:f>
             <x14:dxf>
               <fill>
-                <patternFill>
+                <patternFill patternType="solid">
                   <bgColor rgb="FFFFC7CE"/>
                 </patternFill>
               </fill>
@@ -3118,44 +3201,8 @@
                 <color rgb="FF006100"/>
               </font>
               <fill>
-                <patternFill>
+                <patternFill patternType="solid">
                   <bgColor rgb="FFC6EFCE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="greaterThan" id="{00000000-000E-0000-0500-000003000000}">
-            <xm:f>Assumptions!$B$37</xm:f>
-            <x14:dxf>
-              <font>
-                <color theme="0"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="greaterThan" id="{00000000-000E-0000-0500-000004000000}">
-            <xm:f>Assumptions!$B$37</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FF00B050"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="5" operator="greaterThan" id="{00000000-000E-0000-0500-000005000000}">
-            <xm:f>Assumptions!$B$37</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC7CE"/>
                 </patternFill>
               </fill>
             </x14:dxf>
@@ -3224,7 +3271,7 @@
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f>"Intrinsic Value Per Share | "&amp;TEXT(DCF!B25,"$0.00")</f>
-        <v>Intrinsic Value Per Share | $396.28</v>
+        <v>Intrinsic Value Per Share | $395.95</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
@@ -3236,7 +3283,7 @@
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <f>"Implied Upside / Downside | "&amp;TEXT(DCF!B27,"0.00%")</f>
-        <v>Implied Upside / Downside | -25.59%</v>
+        <v>Implied Upside / Downside | -25.66%</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
@@ -3252,7 +3299,7 @@
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
         <f>"WACC | "&amp;TEXT(Assumptions!B30,"0.00%")</f>
-        <v>WACC | 9.49%</v>
+        <v>WACC | 9.45%</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">

</xml_diff>